<commit_message>
Order lifecycle on staging (14 Oct): test results and tracker update
- docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md: the two
  runs on test.gokesari.com.
  - Run 1: the rider leg was blocked because a 7-shop owner saw only the
    newest shop. Both orders were completed as pickups.
  - Run 2 (after #168): shop switcher, GoKesari rider, pickup code,
    delivery code and door photo, DELIVERED, and the commission and
    delivery charge are correct.
  - Cashfree sandbox only.
- Test results tracker: adds TR-22 and TR-23 (staging), and TR-24
  (production, waits on the owner).
  - Defects D-24 (fixed in #168) and D-25 to D-27 (open): My Orders card
    wording; checkout takes 30-38 s.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjYKXt9b4KzwrT7fa16tNP
</commit_message>
<xml_diff>
--- a/docs/testing/GOKESARI_TEST_RESULTS_TRACKER_2026-10-14.xlsx
+++ b/docs/testing/GOKESARI_TEST_RESULTS_TRACKER_2026-10-14.xlsx
@@ -15,10 +15,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="791-case plan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Runs'!$A$1:$S$23</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Results (detail)'!$A$1:$I$311</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defects'!$A$1:$G$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Not run &amp; gaps'!$A$1:$D$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Runs'!$A$1:$S$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Results (detail)'!$A$1:$I$341</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defects'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Not run &amp; gaps'!$A$1:$D$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'791-case plan'!$A$1:$G$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 14 Oct 2026, 15:00 UTC. Every recorded test run from 22 Sep to 14 Oct 2026: test site (test.gokesari.com), production (gokesari.com) checks, CI / local automated suites and the database-split verifications.</t>
+          <t>As of 14 Oct 2026, 17:45 UTC. Every recorded test run from 22 Sep to 14 Oct 2026: test site (test.gokesari.com), production (gokesari.com) checks, CI / local automated suites and the database-split verifications.</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$23,A9)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A9)</f>
         <v/>
       </c>
     </row>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$23,A10)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A10)</f>
         <v/>
       </c>
     </row>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$23,A11)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A11)</f>
         <v/>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$23,A12)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A12)</f>
         <v/>
       </c>
     </row>
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$23,A13)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A13)</f>
         <v/>
       </c>
     </row>
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B18" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A18)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A18)</f>
         <v/>
       </c>
       <c r="C18" s="7">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="B19" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A19)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A19)</f>
         <v/>
       </c>
       <c r="C19" s="7">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B20" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A20)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A20)</f>
         <v/>
       </c>
       <c r="C20" s="7">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B21" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A21)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A21)</f>
         <v/>
       </c>
       <c r="C21" s="7">
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="B22" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A22)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A22)</f>
         <v/>
       </c>
       <c r="C22" s="7">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B23" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$311,A23)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A23)</f>
         <v/>
       </c>
       <c r="C23" s="7">
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="B28" s="6">
-        <f>COUNTIF(Defects!$E$2:$E$24,A28)</f>
+        <f>COUNTIF(Defects!$E$2:$E$28,A28)</f>
         <v/>
       </c>
     </row>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B29" s="6">
-        <f>COUNTIF(Defects!$E$2:$E$24,A29)</f>
+        <f>COUNTIF(Defects!$E$2:$E$28,A29)</f>
         <v/>
       </c>
     </row>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="B30" s="6">
-        <f>COUNTIF(Defects!$E$2:$E$24,A30)</f>
+        <f>COUNTIF(Defects!$E$2:$E$28,A30)</f>
         <v/>
       </c>
     </row>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B31" s="6">
-        <f>COUNTIF(Defects!$E$2:$E$24,A31)</f>
+        <f>COUNTIF(Defects!$E$2:$E$28,A31)</f>
         <v/>
       </c>
     </row>
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B32" s="6">
-        <f>COUNTIF(Defects!$E$2:$E$24,A32)</f>
+        <f>COUNTIF(Defects!$E$2:$E$28,A32)</f>
         <v/>
       </c>
     </row>
@@ -1702,59 +1702,135 @@
         <v/>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+    <row r="59" ht="27" customHeight="1">
+      <c r="A59" s="5">
+        <f>'Test Runs'!A24&amp;"  "&amp;'Test Runs'!D24</f>
+        <v/>
+      </c>
+      <c r="B59" s="6">
+        <f>'Test Runs'!B24</f>
+        <v/>
+      </c>
+      <c r="C59" s="6">
+        <f>IF('Test Runs'!H24="","-",'Test Runs'!H24)</f>
+        <v/>
+      </c>
+      <c r="D59" s="6">
+        <f>IF('Test Runs'!I24="","-",'Test Runs'!I24)</f>
+        <v/>
+      </c>
+      <c r="E59" s="6">
+        <f>IF('Test Runs'!J24="","-",'Test Runs'!J24)</f>
+        <v/>
+      </c>
+      <c r="F59" s="6">
+        <f>'Test Runs'!L24</f>
+        <v/>
+      </c>
+      <c r="G59" s="6">
+        <f>'Test Runs'!O24</f>
+        <v/>
+      </c>
+      <c r="H59" s="6">
+        <f>'Test Runs'!Q24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="27" customHeight="1">
+      <c r="A60" s="5">
+        <f>'Test Runs'!A25&amp;"  "&amp;'Test Runs'!D25</f>
+        <v/>
+      </c>
+      <c r="B60" s="6">
+        <f>'Test Runs'!B25</f>
+        <v/>
+      </c>
+      <c r="C60" s="6">
+        <f>IF('Test Runs'!H25="","-",'Test Runs'!H25)</f>
+        <v/>
+      </c>
+      <c r="D60" s="6">
+        <f>IF('Test Runs'!I25="","-",'Test Runs'!I25)</f>
+        <v/>
+      </c>
+      <c r="E60" s="6">
+        <f>IF('Test Runs'!J25="","-",'Test Runs'!J25)</f>
+        <v/>
+      </c>
+      <c r="F60" s="6">
+        <f>'Test Runs'!L25</f>
+        <v/>
+      </c>
+      <c r="G60" s="6">
+        <f>'Test Runs'!O25</f>
+        <v/>
+      </c>
+      <c r="H60" s="6">
+        <f>'Test Runs'!Q25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>5. Headlines (14 Oct 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="36" customHeight="1">
-      <c r="A61" s="9" t="inlineStr">
-        <is>
-          <t>1. 22 test runs recorded (310 individual checks). Most features released 8-14 Oct were tested on test.gokesari.com and spot-checked on gokesari.com after release; Seller Central has local checks only and the saffron wordmark change has no recorded run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="36" customHeight="1">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>2. Latest: the seller / customer database split verified PASS on production (14 Oct, run 19: 190 tables, 486 rows, every checksum equal) after the test split (13 Oct). Please confirm the production split databases' names.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="36" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>3. Open defects: OCR auto-read does not start on Hostinger (D-18); mail host hourly cap (D-04); hydration error on /wallet and /admin/orders (D-13); same subquery bug in 3 queries (D-15); stale lifecycle E2E steps (D-20); slow 4G pages (D-07).</t>
+          <t>1. 24 test runs recorded (340 individual checks). Most features released 8-14 Oct were tested on test.gokesari.com and spot-checked on gokesari.com after release; Seller Central was checked on test only through its shop switcher (TR-23), and the saffron wordmark change has no recorded run.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="36" customHeight="1">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>4. Owner actions found by testing: Maps server key restriction (D-05, D-10); Verification Suite keys (D-23); SMS provider for test (D-11).</t>
+          <t>2. Latest: the seller / customer database split verified PASS on production (14 Oct, run 19: 190 tables, 486 rows, every checksum equal) after the test split (13 Oct). Please confirm the production split databases' names.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="36" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>5. Not run yet: the 791-case plan (0 of 791 executed) and the order-lifecycle run on staging (local 21/21 only).</t>
+          <t>3. Open defects: OCR auto-read does not start on Hostinger (D-18); mail host hourly cap (D-04); hydration error on /wallet and /admin/orders (D-13); same subquery bug in 3 queries (D-15); stale lifecycle E2E steps (D-20); slow 4G pages (D-07); slow checkout (D-27).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="36" customHeight="1">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>4. Owner actions found by testing: Maps server key restriction (D-05, D-10); Verification Suite keys (D-23); SMS provider for test (D-11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="36" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>5. Order lifecycle on staging (14 Oct): PASS after #168 (TR-23) - sign-up, sandbox top-up, order, GoKesari rider with pickup code, delivery code and door photo, DELIVERED, commission and delivery charge right. Open: D-25 and D-26 (My Orders card wording), D-27 (checkout 30-38 s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="36" customHeight="1">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>6. Not run yet: the 791-case plan (0 of 791 executed) and the order lifecycle on production (TR-24, waits on the owner).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A67:H67"/>
     <mergeCell ref="A3:H3"/>
     <mergeCell ref="A65:H65"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A63:H63"/>
     <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A66:H66"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A61:H61"/>
   </mergeCells>
   <conditionalFormatting sqref="A9:A13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -1810,7 +1886,7 @@
       <formula>"To confirm"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37:H58">
+  <conditionalFormatting sqref="H37:H60">
     <cfRule type="cellIs" priority="17" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1838,7 +1914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S23"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2008,23 +2084,23 @@
         <v>0</v>
       </c>
       <c r="L2" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A2)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A2)</f>
         <v/>
       </c>
       <c r="M2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A2,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q2" s="6" t="inlineStr">
@@ -2084,23 +2160,23 @@
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A3)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A3)</f>
         <v/>
       </c>
       <c r="M3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A3,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q3" s="6" t="inlineStr">
@@ -2160,23 +2236,23 @@
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A4)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A4)</f>
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A4,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q4" s="6" t="inlineStr">
@@ -2236,23 +2312,23 @@
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A5)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A5)</f>
         <v/>
       </c>
       <c r="M5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A5,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q5" s="6" t="inlineStr">
@@ -2312,23 +2388,23 @@
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A6)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A6)</f>
         <v/>
       </c>
       <c r="M6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A6,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q6" s="6" t="inlineStr">
@@ -2388,23 +2464,23 @@
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A7)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A7)</f>
         <v/>
       </c>
       <c r="M7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A7,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q7" s="6" t="inlineStr">
@@ -2464,23 +2540,23 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A8)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A8)</f>
         <v/>
       </c>
       <c r="M8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A8,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q8" s="6" t="inlineStr">
@@ -2548,23 +2624,23 @@
         <v>4</v>
       </c>
       <c r="L9" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A9)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A9)</f>
         <v/>
       </c>
       <c r="M9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A9,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -2624,23 +2700,23 @@
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A10)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A10)</f>
         <v/>
       </c>
       <c r="M10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A10,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q10" s="6" t="inlineStr">
@@ -2700,23 +2776,23 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A11)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A11)</f>
         <v/>
       </c>
       <c r="M11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A11,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q11" s="6" t="inlineStr">
@@ -2776,23 +2852,23 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A12)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A12)</f>
         <v/>
       </c>
       <c r="M12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A12,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q12" s="6" t="inlineStr">
@@ -2852,23 +2928,23 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A13)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A13)</f>
         <v/>
       </c>
       <c r="M13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A13,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -2928,23 +3004,23 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A14)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A14)</f>
         <v/>
       </c>
       <c r="M14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A14,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q14" s="6" t="inlineStr">
@@ -3004,23 +3080,23 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A15)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A15)</f>
         <v/>
       </c>
       <c r="M15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A15,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q15" s="6" t="inlineStr">
@@ -3080,23 +3156,23 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A16)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A16)</f>
         <v/>
       </c>
       <c r="M16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A16,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q16" s="6" t="inlineStr">
@@ -3156,23 +3232,23 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A17)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A17)</f>
         <v/>
       </c>
       <c r="M17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A17,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q17" s="6" t="inlineStr">
@@ -3232,23 +3308,23 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A18)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A18)</f>
         <v/>
       </c>
       <c r="M18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A18,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q18" s="6" t="inlineStr">
@@ -3316,23 +3392,23 @@
         <v>0</v>
       </c>
       <c r="L19" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A19)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A19)</f>
         <v/>
       </c>
       <c r="M19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A19,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q19" s="6" t="inlineStr">
@@ -3400,23 +3476,23 @@
         <v>0</v>
       </c>
       <c r="L20" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A20)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A20)</f>
         <v/>
       </c>
       <c r="M20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A20,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q20" s="6" t="inlineStr">
@@ -3484,23 +3560,23 @@
         <v>0</v>
       </c>
       <c r="L21" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A21)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A21)</f>
         <v/>
       </c>
       <c r="M21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A21,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q21" s="6" t="inlineStr">
@@ -3568,23 +3644,23 @@
         <v>791</v>
       </c>
       <c r="L22" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A22)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A22)</f>
         <v/>
       </c>
       <c r="M22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A22,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q22" s="6" t="inlineStr">
@@ -3603,7 +3679,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="27" customHeight="1">
+    <row r="23" ht="39" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>TR-22</t>
@@ -3611,32 +3687,32 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>test.gokesari.com</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Order lifecycle on staging, run 1: sign-up -&gt; sandbox top-up -&gt; 2 orders -&gt; pickup / delivery -&gt; DELIVERED</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>QA-008, NEW-039, NEW-007</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>test.gokesari.com</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Order lifecycle on staging: sign-up -&gt; order -&gt; delivery code -&gt; done</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>QA-008</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Browser + Cashfree sandbox</t>
+          <t>API + browser (Chromium), real emailed codes, Cashfree sandbox</t>
         </is>
       </c>
       <c r="H23" s="6" t="n"/>
@@ -3644,44 +3720,196 @@
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$311,A23)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A23)</f>
         <v/>
       </c>
       <c r="M23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"PASS")</f>
         <v/>
       </c>
       <c r="N23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
         <v/>
       </c>
       <c r="P23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$311,A23,'Results (detail)'!$I$2:$I$311,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q23" s="6" t="inlineStr">
         <is>
+          <t>PASS with open items</t>
+        </is>
+      </c>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>Rider leg blocked: a 7-shop owner saw only the newest shop, so the pickup code was not visible (D-24, fixed in #168). Both orders completed as pickups. D-25, D-27 open</t>
+        </is>
+      </c>
+      <c r="S23" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md (Run 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="51" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>test.gokesari.com</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Order lifecycle on staging, run 2 after #168: shop switcher -&gt; order -&gt; GoKesari rider -&gt; pickup code -&gt; delivery code + photo -&gt; DELIVERED -&gt; wallet charges</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>QA-008, NEW-060, NEW-007</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>#168</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>API + browser (Chromium), real emailed codes, Cashfree sandbox</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="6" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6">
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <v/>
+      </c>
+      <c r="O24" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="P24" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <v/>
+      </c>
+      <c r="Q24" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>Full rider delivery works. Still open: D-25, D-26 (My Orders card wording), D-27 (checkout 37.8 s)</t>
+        </is>
+      </c>
+      <c r="S24" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md (Run 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="27" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>TR-24</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>gokesari.com</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Order lifecycle on production with a real payment</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>QA-008</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>API + browser, real payment by the owner</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="6" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6">
+        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <v/>
+      </c>
+      <c r="O25" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="P25" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="6" t="inlineStr">
+        <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="R23" s="6" t="inlineStr">
-        <is>
-          <t>Run locally only (21/21); staging run is next</t>
-        </is>
-      </c>
-      <c r="S23" s="6" t="inlineStr">
-        <is>
-          <t>docs/document-upload-2026-10/TEST_RESULTS.md (Not run yet)</t>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>Waits on the owner: production shop + owner email, approved rider, Cashfree live keys confirmed, owner pays the top-up</t>
+        </is>
+      </c>
+      <c r="S25" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md (Production)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S23"/>
-  <conditionalFormatting sqref="Q2:Q23">
+  <autoFilter ref="A1:S25"/>
+  <conditionalFormatting sqref="Q2:Q25">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -3709,7 +3937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I311"/>
+  <dimension ref="A1:I341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -17508,9 +17736,1415 @@
         </is>
       </c>
     </row>
+    <row r="312" ht="27" customHeight="1">
+      <c r="A312" s="6" t="inlineStr">
+        <is>
+          <t>RES-0311</t>
+        </is>
+      </c>
+      <c r="B312" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C312" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D312" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E312" s="6" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="F312" s="6" t="inlineStr">
+        <is>
+          <t>Sign-up</t>
+        </is>
+      </c>
+      <c r="G312" s="6" t="inlineStr">
+        <is>
+          <t>Sign up by emailed link; profile with mobile; two addresses</t>
+        </is>
+      </c>
+      <c r="H312" s="6" t="inlineStr">
+        <is>
+          <t>Signed in; profile and addresses saved</t>
+        </is>
+      </c>
+      <c r="I312" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="27" customHeight="1">
+      <c r="A313" s="6" t="inlineStr">
+        <is>
+          <t>RES-0312</t>
+        </is>
+      </c>
+      <c r="B313" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C313" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D313" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E313" s="6" t="inlineStr">
+        <is>
+          <t>16:03</t>
+        </is>
+      </c>
+      <c r="F313" s="6" t="inlineStr">
+        <is>
+          <t>Wallet</t>
+        </is>
+      </c>
+      <c r="G313" s="6" t="inlineStr">
+        <is>
+          <t>Top-up Rs 200, Cashfree sandbox UPI (workflow run 38594861540)</t>
+        </is>
+      </c>
+      <c r="H313" s="6" t="inlineStr">
+        <is>
+          <t>Verified; wallet Rs 200</t>
+        </is>
+      </c>
+      <c r="I313" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="27" customHeight="1">
+      <c r="A314" s="6" t="inlineStr">
+        <is>
+          <t>RES-0313</t>
+        </is>
+      </c>
+      <c r="B314" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C314" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D314" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E314" s="6" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="F314" s="6" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="G314" s="6" t="inlineStr">
+        <is>
+          <t>Order 1 DB-20261014-ZQH9MI, bakery, wallet</t>
+        </is>
+      </c>
+      <c r="H314" s="6" t="inlineStr">
+        <is>
+          <t>Timed out at 30 s; retry with the same request id: one order, charged once (D-27)</t>
+        </is>
+      </c>
+      <c r="I314" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="27" customHeight="1">
+      <c r="A315" s="6" t="inlineStr">
+        <is>
+          <t>RES-0314</t>
+        </is>
+      </c>
+      <c r="B315" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C315" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D315" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E315" s="6" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="F315" s="6" t="inlineStr">
+        <is>
+          <t>Shop fulfilment</t>
+        </is>
+      </c>
+      <c r="G315" s="6" t="inlineStr">
+        <is>
+          <t>Accept -&gt; preparing -&gt; GoKesari rider, mark ready</t>
+        </is>
+      </c>
+      <c r="H315" s="6" t="inlineStr">
+        <is>
+          <t>READY; rider offered at once and accepted</t>
+        </is>
+      </c>
+      <c r="I315" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="27" customHeight="1">
+      <c r="A316" s="6" t="inlineStr">
+        <is>
+          <t>RES-0315</t>
+        </is>
+      </c>
+      <c r="B316" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C316" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D316" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E316" s="6" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="F316" s="6" t="inlineStr">
+        <is>
+          <t>Rider pickup</t>
+        </is>
+      </c>
+      <c r="G316" s="6" t="inlineStr">
+        <is>
+          <t>Pickup code on Seller Central -&gt; Orders</t>
+        </is>
+      </c>
+      <c r="H316" s="6" t="inlineStr">
+        <is>
+          <t>Not shown: the 7-shop owner saw only the newest shop (D-24)</t>
+        </is>
+      </c>
+      <c r="I316" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="27" customHeight="1">
+      <c r="A317" s="6" t="inlineStr">
+        <is>
+          <t>RES-0316</t>
+        </is>
+      </c>
+      <c r="B317" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C317" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D317" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E317" s="6" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="F317" s="6" t="inlineStr">
+        <is>
+          <t>Shop fulfilment</t>
+        </is>
+      </c>
+      <c r="G317" s="6" t="inlineStr">
+        <is>
+          <t>Switch order 1 to pickup</t>
+        </is>
+      </c>
+      <c r="H317" s="6" t="inlineStr">
+        <is>
+          <t>Rider released; Rs 20 delivery fee refunded</t>
+        </is>
+      </c>
+      <c r="I317" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="27" customHeight="1">
+      <c r="A318" s="6" t="inlineStr">
+        <is>
+          <t>RES-0317</t>
+        </is>
+      </c>
+      <c r="B318" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C318" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D318" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E318" s="6" t="inlineStr">
+        <is>
+          <t>16:16</t>
+        </is>
+      </c>
+      <c r="F318" s="6" t="inlineStr">
+        <is>
+          <t>Pickup handover</t>
+        </is>
+      </c>
+      <c r="G318" s="6" t="inlineStr">
+        <is>
+          <t>Wrong pickup code, then the right code (8606)</t>
+        </is>
+      </c>
+      <c r="H318" s="6" t="inlineStr">
+        <is>
+          <t>422 '4 attempts left', then DELIVERED; tax invoice</t>
+        </is>
+      </c>
+      <c r="I318" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="27" customHeight="1">
+      <c r="A319" s="6" t="inlineStr">
+        <is>
+          <t>RES-0318</t>
+        </is>
+      </c>
+      <c r="B319" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C319" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D319" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E319" s="6" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="F319" s="6" t="inlineStr">
+        <is>
+          <t>Delivery rule</t>
+        </is>
+      </c>
+      <c r="G319" s="6" t="inlineStr">
+        <is>
+          <t>Order 2 DB-20261014-QS7ZZ5, stationery (delivery off), GoKesari rider</t>
+        </is>
+      </c>
+      <c r="H319" s="6" t="inlineStr">
+        <is>
+          <t>422 'need delivery switched on' - correct</t>
+        </is>
+      </c>
+      <c r="I319" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="27" customHeight="1">
+      <c r="A320" s="6" t="inlineStr">
+        <is>
+          <t>RES-0319</t>
+        </is>
+      </c>
+      <c r="B320" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C320" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D320" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E320" s="6" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="F320" s="6" t="inlineStr">
+        <is>
+          <t>Pickup handover</t>
+        </is>
+      </c>
+      <c r="G320" s="6" t="inlineStr">
+        <is>
+          <t>Order 2 as pickup, code 9246</t>
+        </is>
+      </c>
+      <c r="H320" s="6" t="inlineStr">
+        <is>
+          <t>DELIVERED</t>
+        </is>
+      </c>
+      <c r="I320" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="27" customHeight="1">
+      <c r="A321" s="6" t="inlineStr">
+        <is>
+          <t>RES-0320</t>
+        </is>
+      </c>
+      <c r="B321" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C321" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D321" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E321" s="6" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="F321" s="6" t="inlineStr">
+        <is>
+          <t>Shop wallet</t>
+        </is>
+      </c>
+      <c r="G321" s="6" t="inlineStr">
+        <is>
+          <t>1% commission per order; no delivery charge on pickups</t>
+        </is>
+      </c>
+      <c r="H321" s="6" t="inlineStr">
+        <is>
+          <t>As expected</t>
+        </is>
+      </c>
+      <c r="I321" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="27" customHeight="1">
+      <c r="A322" s="6" t="inlineStr">
+        <is>
+          <t>RES-0321</t>
+        </is>
+      </c>
+      <c r="B322" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C322" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D322" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E322" s="6" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="F322" s="6" t="inlineStr">
+        <is>
+          <t>Emails</t>
+        </is>
+      </c>
+      <c r="G322" s="6" t="inlineStr">
+        <is>
+          <t>Customer emails for each step</t>
+        </is>
+      </c>
+      <c r="H322" s="6" t="inlineStr">
+        <is>
+          <t>All received</t>
+        </is>
+      </c>
+      <c r="I322" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="27" customHeight="1">
+      <c r="A323" s="6" t="inlineStr">
+        <is>
+          <t>RES-0322</t>
+        </is>
+      </c>
+      <c r="B323" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C323" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D323" s="6" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="E323" s="6" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="F323" s="6" t="inlineStr">
+        <is>
+          <t>My Orders</t>
+        </is>
+      </c>
+      <c r="G323" s="6" t="inlineStr">
+        <is>
+          <t>Order 1 card after the switch to pickup</t>
+        </is>
+      </c>
+      <c r="H323" s="6" t="inlineStr">
+        <is>
+          <t>Still 'Finding a rider - E2E Rider Vijay' (D-25)</t>
+        </is>
+      </c>
+      <c r="I323" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="27" customHeight="1">
+      <c r="A324" s="6" t="inlineStr">
+        <is>
+          <t>RES-0323</t>
+        </is>
+      </c>
+      <c r="B324" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C324" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D324" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E324" s="6" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="F324" s="6" t="inlineStr">
+        <is>
+          <t>Seller Central</t>
+        </is>
+      </c>
+      <c r="G324" s="6" t="inlineStr">
+        <is>
+          <t>Shop switcher for the 7-shop owner</t>
+        </is>
+      </c>
+      <c r="H324" s="6" t="inlineStr">
+        <is>
+          <t>Switcher with all 7 shops</t>
+        </is>
+      </c>
+      <c r="I324" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="27" customHeight="1">
+      <c r="A325" s="6" t="inlineStr">
+        <is>
+          <t>RES-0324</t>
+        </is>
+      </c>
+      <c r="B325" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C325" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D325" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E325" s="6" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="F325" s="6" t="inlineStr">
+        <is>
+          <t>Seller Central</t>
+        </is>
+      </c>
+      <c r="G325" s="6" t="inlineStr">
+        <is>
+          <t>Choose the bakery; reload</t>
+        </is>
+      </c>
+      <c r="H325" s="6" t="inlineStr">
+        <is>
+          <t>Bakery shown and kept after reload (cookie gk_shop: Secure, HttpOnly, Lax)</t>
+        </is>
+      </c>
+      <c r="I325" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="27" customHeight="1">
+      <c r="A326" s="6" t="inlineStr">
+        <is>
+          <t>RES-0325</t>
+        </is>
+      </c>
+      <c r="B326" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C326" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D326" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E326" s="6" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="F326" s="6" t="inlineStr">
+        <is>
+          <t>Wallet</t>
+        </is>
+      </c>
+      <c r="G326" s="6" t="inlineStr">
+        <is>
+          <t>Top-up Rs 200, Cashfree sandbox UPI (workflow run 38607067429)</t>
+        </is>
+      </c>
+      <c r="H326" s="6" t="inlineStr">
+        <is>
+          <t>Verified; wallet Rs 20 -&gt; Rs 220</t>
+        </is>
+      </c>
+      <c r="I326" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="27" customHeight="1">
+      <c r="A327" s="6" t="inlineStr">
+        <is>
+          <t>RES-0326</t>
+        </is>
+      </c>
+      <c r="B327" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C327" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D327" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E327" s="6" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="F327" s="6" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="G327" s="6" t="inlineStr">
+        <is>
+          <t>Order 3 DB-20261014-QKJX67, bakery, Rs 80 + Rs 20 delivery, wallet</t>
+        </is>
+      </c>
+      <c r="H327" s="6" t="inlineStr">
+        <is>
+          <t>Placed (Rs 100); wallet Rs 220 -&gt; Rs 120; took 37.8 s (D-27)</t>
+        </is>
+      </c>
+      <c r="I327" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="27" customHeight="1">
+      <c r="A328" s="6" t="inlineStr">
+        <is>
+          <t>RES-0327</t>
+        </is>
+      </c>
+      <c r="B328" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C328" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D328" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E328" s="6" t="inlineStr">
+        <is>
+          <t>17:33</t>
+        </is>
+      </c>
+      <c r="F328" s="6" t="inlineStr">
+        <is>
+          <t>Seller Central</t>
+        </is>
+      </c>
+      <c r="G328" s="6" t="inlineStr">
+        <is>
+          <t>Order on the bakery's Orders page</t>
+        </is>
+      </c>
+      <c r="H328" s="6" t="inlineStr">
+        <is>
+          <t>Shown</t>
+        </is>
+      </c>
+      <c r="I328" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="27" customHeight="1">
+      <c r="A329" s="6" t="inlineStr">
+        <is>
+          <t>RES-0328</t>
+        </is>
+      </c>
+      <c r="B329" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C329" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D329" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E329" s="6" t="inlineStr">
+        <is>
+          <t>17:34</t>
+        </is>
+      </c>
+      <c r="F329" s="6" t="inlineStr">
+        <is>
+          <t>Shop fulfilment</t>
+        </is>
+      </c>
+      <c r="G329" s="6" t="inlineStr">
+        <is>
+          <t>Accept -&gt; preparing -&gt; GoKesari rider, slot Thu 7-8 am, mark ready</t>
+        </is>
+      </c>
+      <c r="H329" s="6" t="inlineStr">
+        <is>
+          <t>READY; rider search scheduled for the slot's lead time</t>
+        </is>
+      </c>
+      <c r="I329" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="27" customHeight="1">
+      <c r="A330" s="6" t="inlineStr">
+        <is>
+          <t>RES-0329</t>
+        </is>
+      </c>
+      <c r="B330" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C330" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D330" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E330" s="6" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="F330" s="6" t="inlineStr">
+        <is>
+          <t>Rider dispatch</t>
+        </is>
+      </c>
+      <c r="G330" s="6" t="inlineStr">
+        <is>
+          <t>Shop presses 'find a rider now'</t>
+        </is>
+      </c>
+      <c r="H330" s="6" t="inlineStr">
+        <is>
+          <t>Rider offered</t>
+        </is>
+      </c>
+      <c r="I330" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="27" customHeight="1">
+      <c r="A331" s="6" t="inlineStr">
+        <is>
+          <t>RES-0330</t>
+        </is>
+      </c>
+      <c r="B331" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C331" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D331" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E331" s="6" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="F331" s="6" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="G331" s="6" t="inlineStr">
+        <is>
+          <t>Rider accepts, arrives at the shop</t>
+        </is>
+      </c>
+      <c r="H331" s="6" t="inlineStr">
+        <is>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="I331" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="27" customHeight="1">
+      <c r="A332" s="6" t="inlineStr">
+        <is>
+          <t>RES-0331</t>
+        </is>
+      </c>
+      <c r="B332" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C332" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D332" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E332" s="6" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="F332" s="6" t="inlineStr">
+        <is>
+          <t>Rider pickup</t>
+        </is>
+      </c>
+      <c r="G332" s="6" t="inlineStr">
+        <is>
+          <t>Pickup code on the bakery's Orders page</t>
+        </is>
+      </c>
+      <c r="H332" s="6" t="inlineStr">
+        <is>
+          <t>Shown (4584) - D-24 fixed</t>
+        </is>
+      </c>
+      <c r="I332" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="27" customHeight="1">
+      <c r="A333" s="6" t="inlineStr">
+        <is>
+          <t>RES-0332</t>
+        </is>
+      </c>
+      <c r="B333" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C333" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D333" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E333" s="6" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="F333" s="6" t="inlineStr">
+        <is>
+          <t>Rider pickup</t>
+        </is>
+      </c>
+      <c r="G333" s="6" t="inlineStr">
+        <is>
+          <t>Wrong pickup code, then the right one</t>
+        </is>
+      </c>
+      <c r="H333" s="6" t="inlineStr">
+        <is>
+          <t>422, then PICKED_UP</t>
+        </is>
+      </c>
+      <c r="I333" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="27" customHeight="1">
+      <c r="A334" s="6" t="inlineStr">
+        <is>
+          <t>RES-0333</t>
+        </is>
+      </c>
+      <c r="B334" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C334" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D334" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E334" s="6" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="F334" s="6" t="inlineStr">
+        <is>
+          <t>Delivery code</t>
+        </is>
+      </c>
+      <c r="G334" s="6" t="inlineStr">
+        <is>
+          <t>Rider starts and arrives; delivery code email; ask again</t>
+        </is>
+      </c>
+      <c r="H334" s="6" t="inlineStr">
+        <is>
+          <t>Code emailed (0598); ask again refused in the 40 s cool-down (429)</t>
+        </is>
+      </c>
+      <c r="I334" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="27" customHeight="1">
+      <c r="A335" s="6" t="inlineStr">
+        <is>
+          <t>RES-0334</t>
+        </is>
+      </c>
+      <c r="B335" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C335" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D335" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E335" s="6" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="F335" s="6" t="inlineStr">
+        <is>
+          <t>Proof photo</t>
+        </is>
+      </c>
+      <c r="G335" s="6" t="inlineStr">
+        <is>
+          <t>Mark delivered without a photo</t>
+        </is>
+      </c>
+      <c r="H335" s="6" t="inlineStr">
+        <is>
+          <t>409 'Take a photo of the order at the door'</t>
+        </is>
+      </c>
+      <c r="I335" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="27" customHeight="1">
+      <c r="A336" s="6" t="inlineStr">
+        <is>
+          <t>RES-0335</t>
+        </is>
+      </c>
+      <c r="B336" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C336" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D336" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E336" s="6" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="F336" s="6" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="G336" s="6" t="inlineStr">
+        <is>
+          <t>Upload door photo; wrong code; right code</t>
+        </is>
+      </c>
+      <c r="H336" s="6" t="inlineStr">
+        <is>
+          <t>201; 422 '4 attempts left'; DELIVERED 17:38:18</t>
+        </is>
+      </c>
+      <c r="I336" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="27" customHeight="1">
+      <c r="A337" s="6" t="inlineStr">
+        <is>
+          <t>RES-0336</t>
+        </is>
+      </c>
+      <c r="B337" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C337" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D337" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E337" s="6" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="F337" s="6" t="inlineStr">
+        <is>
+          <t>Shop wallet</t>
+        </is>
+      </c>
+      <c r="G337" s="6" t="inlineStr">
+        <is>
+          <t>Commission and delivery charge</t>
+        </is>
+      </c>
+      <c r="H337" s="6" t="inlineStr">
+        <is>
+          <t>Rs 0.80 (1% of Rs 80) + Rs 7.50 (1.51 km at Rs 5/km): Rs 965.70 -&gt; Rs 957.40</t>
+        </is>
+      </c>
+      <c r="I337" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="27" customHeight="1">
+      <c r="A338" s="6" t="inlineStr">
+        <is>
+          <t>RES-0337</t>
+        </is>
+      </c>
+      <c r="B338" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C338" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D338" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E338" s="6" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="F338" s="6" t="inlineStr">
+        <is>
+          <t>My Orders</t>
+        </is>
+      </c>
+      <c r="G338" s="6" t="inlineStr">
+        <is>
+          <t>Order 3 card</t>
+        </is>
+      </c>
+      <c r="H338" s="6" t="inlineStr">
+        <is>
+          <t>DELIVERED, Rs 100, tax invoice, photo at delivery</t>
+        </is>
+      </c>
+      <c r="I338" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="27" customHeight="1">
+      <c r="A339" s="6" t="inlineStr">
+        <is>
+          <t>RES-0338</t>
+        </is>
+      </c>
+      <c r="B339" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C339" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D339" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E339" s="6" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="F339" s="6" t="inlineStr">
+        <is>
+          <t>Rider</t>
+        </is>
+      </c>
+      <c r="G339" s="6" t="inlineStr">
+        <is>
+          <t>Rider offline</t>
+        </is>
+      </c>
+      <c r="H339" s="6" t="inlineStr">
+        <is>
+          <t>Offline</t>
+        </is>
+      </c>
+      <c r="I339" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="27" customHeight="1">
+      <c r="A340" s="6" t="inlineStr">
+        <is>
+          <t>RES-0339</t>
+        </is>
+      </c>
+      <c r="B340" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C340" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D340" s="6" t="inlineStr">
+        <is>
+          <t>Run 2</t>
+        </is>
+      </c>
+      <c r="E340" s="6" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="F340" s="6" t="inlineStr">
+        <is>
+          <t>My Orders</t>
+        </is>
+      </c>
+      <c r="G340" s="6" t="inlineStr">
+        <is>
+          <t>Order 1 card (pickup, delivered)</t>
+        </is>
+      </c>
+      <c r="H340" s="6" t="inlineStr">
+        <is>
+          <t>'Finding a rider' still shown (D-25); delivery-fee refund labelled 'for unavailable items' (D-26)</t>
+        </is>
+      </c>
+      <c r="I340" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="27" customHeight="1">
+      <c r="A341" s="6" t="inlineStr">
+        <is>
+          <t>RES-0340</t>
+        </is>
+      </c>
+      <c r="B341" s="6" t="inlineStr">
+        <is>
+          <t>TR-24</t>
+        </is>
+      </c>
+      <c r="C341" s="6" t="inlineStr">
+        <is>
+          <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md</t>
+        </is>
+      </c>
+      <c r="D341" s="6" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="E341" s="6" t="inlineStr"/>
+      <c r="F341" s="6" t="inlineStr">
+        <is>
+          <t>Production lifecycle</t>
+        </is>
+      </c>
+      <c r="G341" s="6" t="inlineStr">
+        <is>
+          <t>Full order with a real payment on gokesari.com</t>
+        </is>
+      </c>
+      <c r="H341" s="6" t="inlineStr">
+        <is>
+          <t>Waits on the owner's shop, rider, live keys and payment</t>
+        </is>
+      </c>
+      <c r="I341" s="6" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I311"/>
-  <conditionalFormatting sqref="I2:I311">
+  <autoFilter ref="A1:I341"/>
+  <conditionalFormatting sqref="I2:I341">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -17531,7 +19165,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I311" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I2:I341" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"PASS,OK (recorded),FAIL,BLOCKED,NOT RUN,ISSUE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17546,7 +19180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -18446,9 +20080,157 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="27" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>D-24</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>NEW-060</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>An owner with several shops saw only the newest shop in Seller Central: other shops' orders and the rider pickup code were not visible</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>#168</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Shop switcher; re-checked in TR-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="27" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D-25</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>NEW-039</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>My Orders still shows 'Finding a rider - &lt;rider&gt;' after the shop changed the order to pickup and it was delivered</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Re-seen in TR-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="27" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D-26</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>TR-23</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>NEW-039</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>My Orders labels the pickup delivery-fee refund (Rs 20) 'refunded to your wallet for unavailable items'</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Wording only; the refund amount is right</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="27" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>D-27</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>TR-22</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>GS-029</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Wallet checkout takes 30-38 s on test (one call timed out at 30 s; the retry was safe and charged once)</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>Re-seen in TR-23 (37.8 s); likely the far database (see D-07)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G24"/>
-  <conditionalFormatting sqref="E2:E24">
+  <autoFilter ref="A1:G28"/>
+  <conditionalFormatting sqref="E2:E28">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Fixed"</formula>
     </cfRule>
@@ -18476,7 +20258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -18532,7 +20314,7 @@
     <row r="3" ht="27" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Order lifecycle on staging (sign-up -&gt; order -&gt; delivery code -&gt; done)</t>
+          <t>Order lifecycle on production with a real payment</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -18542,51 +20324,51 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Run locally only (21/21); staging run is next and needs the Sandbox payment workflow</t>
+          <t>Waits on the owner: production shop + owner email, approved rider, Cashfree live keys, owner pays the top-up</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>TR-22</t>
+          <t>TR-24</t>
         </is>
       </c>
     </row>
     <row r="4" ht="27" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>Shop's own delivery person (SHOP_DELIVERY) in the staging lifecycle</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>NEW-039</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not part of the 14 Oct runs (pickup and GoKesari rider were run)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Integration tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
           <t>Shop settlement refused without a verified bank account</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>NEW-041</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>No settlement can exist on test for a new shop until the hold period passes</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Integration tests</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Payer-name mismatch on the Rs 1 payment</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>NEW-041</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Cashfree sandbox reports no payer name</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -18598,149 +20380,149 @@
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Arrival of request emails in the referrals@gokesari.com inbox</t>
+          <t>Payer-name mismatch on the Rs 1 payment</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>NEW-042</t>
+          <t>NEW-041</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Mailbox not readable from the test run (SMTP accepted)</t>
+          <t>Cashfree sandbox reports no payer name</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Owner to confirm</t>
+          <t>Integration tests</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>Arrival of request emails in the referrals@gokesari.com inbox</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>NEW-042</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Mailbox not readable from the test run (SMTP accepted)</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Owner to confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
           <t>Paid self-registration (/shop/join) end to end</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>NEW-038, NEW-058</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>No SMS provider on test (N-2)</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Integration tests</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="27" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="9" ht="27" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Wallet top-up and shop wallet recharge in the UI pass (C-01, S-13)</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>GS-029, NEW-033</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>GitHub Actions billing stop on 9 Oct (Sandbox payment did not start)</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Covered in TR-02 and TR-10 regression</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Return pickup, inspection and refund (S-11b)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>GS-057</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Needs a rider to collect the pickup</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Seller Central on test / production</t>
+          <t>Return pickup, inspection and refund (S-11b)</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>NEW-060</t>
+          <t>GS-057</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Only local checks recorded</t>
+          <t>Needs a rider to collect the pickup</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>TR-13</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Saffron wordmark (#153) on test / production</t>
+          <t>Seller Central on production; full Seller Central pass on test</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>NEW-064</t>
+          <t>NEW-060</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>No run recorded after the change</t>
+          <t>Local checks (TR-13) and the shop switcher on test (TR-23) only</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TR-13, TR-23</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Directions on a real phone</t>
+          <t>Saffron wordmark (#153) on test / production</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>NEW-057</t>
+          <t>NEW-064</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Test environment cannot reach google.com</t>
+          <t>No run recorded after the change</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -18752,49 +20534,71 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>Directions on a real phone</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>NEW-057</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Test environment cannot reach google.com</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
           <t>Firefox and Safari</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Only Chromium available in the test sessions</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="27" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15" ht="27" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Admin pages on production (referral settings, referral-code counts)</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>NEW-058, NEW-065</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Need a production admin sign-in</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Verified on test</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D14"/>
+  <autoFilter ref="A1:D15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Staging: #169 test results and trackers (as merged to main in #178)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBjybK9TNUiDeHR27XPHU
</commit_message>
<xml_diff>
--- a/docs/testing/GOKESARI_TEST_RESULTS_TRACKER_2026-10-14.xlsx
+++ b/docs/testing/GOKESARI_TEST_RESULTS_TRACKER_2026-10-14.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -581,7 +581,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 14 Oct 2026, 17:45 UTC. Every recorded test run from 22 Sep to 14 Oct 2026: test site (test.gokesari.com), production (gokesari.com) checks, CI / local automated suites and the database-split verifications.</t>
+          <t>As of 15 Oct 2026, 15:00 UTC. Every recorded test run from 22 Sep to 15 Oct 2026: test site (test.gokesari.com), production (gokesari.com) checks, CI / local automated suites and the database-split verifications.</t>
         </is>
       </c>
     </row>
@@ -606,6 +606,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -632,7 +633,7 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A9)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$60,A9)</f>
         <v/>
       </c>
     </row>
@@ -643,7 +644,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A10)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$60,A10)</f>
         <v/>
       </c>
     </row>
@@ -654,7 +655,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A11)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$60,A11)</f>
         <v/>
       </c>
     </row>
@@ -665,7 +666,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A12)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$60,A12)</f>
         <v/>
       </c>
     </row>
@@ -676,7 +677,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIF('Test Runs'!$Q$2:$Q$25,A13)</f>
+        <f>COUNTIF('Test Runs'!$Q$2:$Q$60,A13)</f>
         <v/>
       </c>
     </row>
@@ -691,6 +692,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -722,7 +724,7 @@
         </is>
       </c>
       <c r="B18" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A18)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A18)</f>
         <v/>
       </c>
       <c r="C18" s="7">
@@ -737,7 +739,7 @@
         </is>
       </c>
       <c r="B19" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A19)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A19)</f>
         <v/>
       </c>
       <c r="C19" s="7">
@@ -752,7 +754,7 @@
         </is>
       </c>
       <c r="B20" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A20)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A20)</f>
         <v/>
       </c>
       <c r="C20" s="7">
@@ -767,7 +769,7 @@
         </is>
       </c>
       <c r="B21" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A21)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A21)</f>
         <v/>
       </c>
       <c r="C21" s="7">
@@ -782,7 +784,7 @@
         </is>
       </c>
       <c r="B22" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A22)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A22)</f>
         <v/>
       </c>
       <c r="C22" s="7">
@@ -797,7 +799,7 @@
         </is>
       </c>
       <c r="B23" s="6">
-        <f>COUNTIF('Results (detail)'!$I$2:$I$341,A23)</f>
+        <f>COUNTIF('Results (detail)'!$I$2:$I$500,A23)</f>
         <v/>
       </c>
       <c r="C23" s="7">
@@ -820,6 +822,7 @@
         <v/>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -905,6 +908,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
@@ -1770,64 +1774,167 @@
         <v/>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>5. Headlines (14 Oct 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="36" customHeight="1">
-      <c r="A63" s="9" t="inlineStr">
-        <is>
-          <t>1. 24 test runs recorded (340 individual checks). Most features released 8-14 Oct were tested on test.gokesari.com and spot-checked on gokesari.com after release; Seller Central was checked on test only through its shop switcher (TR-23), and the saffron wordmark change has no recorded run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="36" customHeight="1">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>2. Latest: the seller / customer database split verified PASS on production (14 Oct, run 19: 190 tables, 486 rows, every checksum equal) after the test split (13 Oct). Please confirm the production split databases' names.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="36" customHeight="1">
-      <c r="A65" s="9" t="inlineStr">
-        <is>
-          <t>3. Open defects: OCR auto-read does not start on Hostinger (D-18); mail host hourly cap (D-04); hydration error on /wallet and /admin/orders (D-13); same subquery bug in 3 queries (D-15); stale lifecycle E2E steps (D-20); slow 4G pages (D-07); slow checkout (D-27).</t>
+    <row r="61" ht="27" customHeight="1">
+      <c r="A61" s="5">
+        <f>'Test Runs'!A26&amp;"  "&amp;'Test Runs'!D26</f>
+        <v/>
+      </c>
+      <c r="B61" s="6">
+        <f>'Test Runs'!B26</f>
+        <v/>
+      </c>
+      <c r="C61" s="6">
+        <f>IF('Test Runs'!H26="","-",'Test Runs'!H26)</f>
+        <v/>
+      </c>
+      <c r="D61" s="6">
+        <f>IF('Test Runs'!I26="","-",'Test Runs'!I26)</f>
+        <v/>
+      </c>
+      <c r="E61" s="6">
+        <f>IF('Test Runs'!J26="","-",'Test Runs'!J26)</f>
+        <v/>
+      </c>
+      <c r="F61" s="6">
+        <f>'Test Runs'!L26</f>
+        <v/>
+      </c>
+      <c r="G61" s="6">
+        <f>'Test Runs'!O26</f>
+        <v/>
+      </c>
+      <c r="H61" s="6">
+        <f>'Test Runs'!Q26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="27" customHeight="1">
+      <c r="A62" s="5">
+        <f>'Test Runs'!A27&amp;"  "&amp;'Test Runs'!D27</f>
+        <v/>
+      </c>
+      <c r="B62" s="6">
+        <f>'Test Runs'!B27</f>
+        <v/>
+      </c>
+      <c r="C62" s="6">
+        <f>IF('Test Runs'!H27="","-",'Test Runs'!H27)</f>
+        <v/>
+      </c>
+      <c r="D62" s="6">
+        <f>IF('Test Runs'!I27="","-",'Test Runs'!I27)</f>
+        <v/>
+      </c>
+      <c r="E62" s="6">
+        <f>IF('Test Runs'!J27="","-",'Test Runs'!J27)</f>
+        <v/>
+      </c>
+      <c r="F62" s="6">
+        <f>'Test Runs'!L27</f>
+        <v/>
+      </c>
+      <c r="G62" s="6">
+        <f>'Test Runs'!O27</f>
+        <v/>
+      </c>
+      <c r="H62" s="6">
+        <f>'Test Runs'!Q27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="27" customHeight="1">
+      <c r="A63" s="5">
+        <f>'Test Runs'!A28&amp;"  "&amp;'Test Runs'!D28</f>
+        <v/>
+      </c>
+      <c r="B63" s="6">
+        <f>'Test Runs'!B28</f>
+        <v/>
+      </c>
+      <c r="C63" s="6">
+        <f>IF('Test Runs'!H28="","-",'Test Runs'!H28)</f>
+        <v/>
+      </c>
+      <c r="D63" s="6">
+        <f>IF('Test Runs'!I28="","-",'Test Runs'!I28)</f>
+        <v/>
+      </c>
+      <c r="E63" s="6">
+        <f>IF('Test Runs'!J28="","-",'Test Runs'!J28)</f>
+        <v/>
+      </c>
+      <c r="F63" s="6">
+        <f>'Test Runs'!L28</f>
+        <v/>
+      </c>
+      <c r="G63" s="6">
+        <f>'Test Runs'!O28</f>
+        <v/>
+      </c>
+      <c r="H63" s="6">
+        <f>'Test Runs'!Q28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64"/>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>5. Headlines (15 Oct 2026)</t>
         </is>
       </c>
     </row>
     <row r="66" ht="36" customHeight="1">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>4. Owner actions found by testing: Maps server key restriction (D-05, D-10); Verification Suite keys (D-23); SMS provider for test (D-11).</t>
+          <t>1. 27 test runs recorded (362 individual checks). Most features released 8-14 Oct were tested on test.gokesari.com and spot-checked on gokesari.com after release; Seller Central was checked on test only through its shop switcher (TR-23), and the saffron wordmark change has no recorded run.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="36" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>5. Order lifecycle on staging (14 Oct): PASS after #168 (TR-23) - sign-up, sandbox top-up, order, GoKesari rider with pickup code, delivery code and door photo, DELIVERED, commission and delivery charge right. Open: D-25 and D-26 (My Orders card wording), D-27 (checkout 30-38 s).</t>
+          <t>2. Latest: the seller / customer database split verified PASS on production (14 Oct, run 19: 190 tables, 486 rows, every checksum equal) after the test split (13 Oct). Please confirm the production split databases' names.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="36" customHeight="1">
       <c r="A68" s="9" t="inlineStr">
         <is>
+          <t>3. Open defects: mail host hourly cap (D-04); hydration error on /wallet and /admin/orders (D-13); same subquery bug in 3 queries (D-15); stale lifecycle E2E steps (D-20); slow 4G pages (D-07); slow checkout (D-27). D-18 (OCR on Hostinger) was fixed on 15 Oct by reading photos in the owner's browser (#169; TR-26 on test, TR-27 on production).</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="36" customHeight="1">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>4. Owner actions found by testing: Maps server key restriction (D-05, D-10); Verification Suite keys (D-23); SMS provider for test (D-11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="36" customHeight="1">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>5. Order lifecycle on staging (14 Oct): PASS after #168 (TR-23) - sign-up, sandbox top-up, order, GoKesari rider with pickup code, delivery code and door photo, DELIVERED, commission and delivery charge right. Open: D-25 and D-26 (My Orders card wording), D-27 (checkout 30-38 s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="36" customHeight="1">
+      <c r="A71" s="9" t="inlineStr">
+        <is>
           <t>6. Not run yet: the 791-case plan (0 of 791 executed) and the order lifecycle on production (TR-24, waits on the owner).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A70:H70"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A67:H67"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A69:H69"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A63:H63"/>
-    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A71:H71"/>
     <mergeCell ref="A68:H68"/>
     <mergeCell ref="A66:H66"/>
     <mergeCell ref="A5:H5"/>
@@ -1914,7 +2021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2084,23 +2191,23 @@
         <v>0</v>
       </c>
       <c r="L2" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A2)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A2)</f>
         <v/>
       </c>
       <c r="M2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P2" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A2,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A2,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q2" s="6" t="inlineStr">
@@ -2160,23 +2267,23 @@
       <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="n"/>
       <c r="L3" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A3)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A3)</f>
         <v/>
       </c>
       <c r="M3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P3" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A3,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A3,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q3" s="6" t="inlineStr">
@@ -2236,23 +2343,23 @@
       <c r="J4" s="6" t="n"/>
       <c r="K4" s="6" t="n"/>
       <c r="L4" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A4)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A4)</f>
         <v/>
       </c>
       <c r="M4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P4" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A4,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A4,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q4" s="6" t="inlineStr">
@@ -2312,23 +2419,23 @@
       <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="n"/>
       <c r="L5" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A5)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A5)</f>
         <v/>
       </c>
       <c r="M5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P5" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A5,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A5,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q5" s="6" t="inlineStr">
@@ -2388,23 +2495,23 @@
       <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="n"/>
       <c r="L6" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A6)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A6)</f>
         <v/>
       </c>
       <c r="M6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P6" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A6,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A6,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q6" s="6" t="inlineStr">
@@ -2464,23 +2571,23 @@
       <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="n"/>
       <c r="L7" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A7)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A7)</f>
         <v/>
       </c>
       <c r="M7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P7" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A7,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A7,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q7" s="6" t="inlineStr">
@@ -2540,23 +2647,23 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A8)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A8)</f>
         <v/>
       </c>
       <c r="M8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P8" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A8,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A8,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q8" s="6" t="inlineStr">
@@ -2624,23 +2731,23 @@
         <v>4</v>
       </c>
       <c r="L9" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A9)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A9)</f>
         <v/>
       </c>
       <c r="M9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P9" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A9,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A9,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q9" s="6" t="inlineStr">
@@ -2700,23 +2807,23 @@
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A10)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A10)</f>
         <v/>
       </c>
       <c r="M10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P10" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A10,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A10,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q10" s="6" t="inlineStr">
@@ -2776,23 +2883,23 @@
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
       <c r="L11" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A11)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A11)</f>
         <v/>
       </c>
       <c r="M11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P11" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A11,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A11,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q11" s="6" t="inlineStr">
@@ -2852,23 +2959,23 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A12)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A12)</f>
         <v/>
       </c>
       <c r="M12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P12" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A12,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A12,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q12" s="6" t="inlineStr">
@@ -2928,23 +3035,23 @@
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
       <c r="L13" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A13)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A13)</f>
         <v/>
       </c>
       <c r="M13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P13" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A13,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A13,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q13" s="6" t="inlineStr">
@@ -3004,23 +3111,23 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A14)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A14)</f>
         <v/>
       </c>
       <c r="M14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P14" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A14,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A14,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q14" s="6" t="inlineStr">
@@ -3080,23 +3187,23 @@
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
       <c r="L15" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A15)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A15)</f>
         <v/>
       </c>
       <c r="M15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P15" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A15,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A15,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q15" s="6" t="inlineStr">
@@ -3156,23 +3263,23 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A16)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A16)</f>
         <v/>
       </c>
       <c r="M16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P16" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A16,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A16,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q16" s="6" t="inlineStr">
@@ -3232,23 +3339,23 @@
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
       <c r="L17" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A17)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A17)</f>
         <v/>
       </c>
       <c r="M17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P17" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A17,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A17,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q17" s="6" t="inlineStr">
@@ -3308,23 +3415,23 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A18)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A18)</f>
         <v/>
       </c>
       <c r="M18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P18" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A18,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A18,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q18" s="6" t="inlineStr">
@@ -3392,23 +3499,23 @@
         <v>0</v>
       </c>
       <c r="L19" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A19)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A19)</f>
         <v/>
       </c>
       <c r="M19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P19" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A19,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A19,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q19" s="6" t="inlineStr">
@@ -3476,23 +3583,23 @@
         <v>0</v>
       </c>
       <c r="L20" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A20)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A20)</f>
         <v/>
       </c>
       <c r="M20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P20" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A20,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A20,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q20" s="6" t="inlineStr">
@@ -3560,23 +3667,23 @@
         <v>0</v>
       </c>
       <c r="L21" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A21)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A21)</f>
         <v/>
       </c>
       <c r="M21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P21" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A21,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A21,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q21" s="6" t="inlineStr">
@@ -3644,23 +3751,23 @@
         <v>791</v>
       </c>
       <c r="L22" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A22)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A22)</f>
         <v/>
       </c>
       <c r="M22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P22" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A22,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A22,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q22" s="6" t="inlineStr">
@@ -3720,23 +3827,23 @@
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A23)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A23)</f>
         <v/>
       </c>
       <c r="M23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P23" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A23,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A23,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q23" s="6" t="inlineStr">
@@ -3796,23 +3903,23 @@
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A24)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A24)</f>
         <v/>
       </c>
       <c r="M24" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N24" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O24" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P24" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A24,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A24,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q24" s="6" t="inlineStr">
@@ -3872,23 +3979,23 @@
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6">
-        <f>COUNTIF('Results (detail)'!$B$2:$B$341,A25)</f>
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A25)</f>
         <v/>
       </c>
       <c r="M25" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"PASS")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"PASS")</f>
         <v/>
       </c>
       <c r="N25" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"OK (recorded)")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
         <v/>
       </c>
       <c r="O25" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"FAIL")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
         <v/>
       </c>
       <c r="P25" s="6">
-        <f>COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$341,A25,'Results (detail)'!$I$2:$I$341,"ISSUE")</f>
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A25,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
         <v/>
       </c>
       <c r="Q25" s="6" t="inlineStr">
@@ -3904,6 +4011,242 @@
       <c r="S25" s="6" t="inlineStr">
         <is>
           <t>docs/order-lifecycle-2026-10/TEST_RESULTS_STAGING_2026-10-14.md (Production)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>CI + local production build</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Browser document reading (#169): automated suites and local browser flow</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>#169</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>Automated (vitest, real PostgreSQL), Playwright E2E on a local production build (desktop + Pixel 7)</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>1762</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>1762</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6">
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"PASS")</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
+        <v/>
+      </c>
+      <c r="O26" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="P26" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A26,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>Two lifecycle steps already stale before this work (D-20) left out, as on 13 Oct</t>
+        </is>
+      </c>
+      <c r="S26" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md (14-15 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>test.gokesari.com</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Browser document reading on staging: baseline before #169, then after the deploy</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>#169</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Browser (Chromium, desktop + Pixel 7), real emailed codes; FSSAI photo on E2E Four Features Bakery, read then discarded (not submitted)</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6">
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"PASS")</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
+        <v/>
+      </c>
+      <c r="O27" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="P27" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A27,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>Baseline (14 Oct) reproduced D-18; after #169 fields pre-filled. First read after the deploy took 25 s (cold start), later 7-8 s</t>
+        </is>
+      </c>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md (15 Oct, staging)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>gokesari.com</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Browser document reading on production (#175 / #177), read-only</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>#175, #177</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>HTTP checks; the reader run in Chromium on a public page from the site's own files (no sign-in, nothing uploaded); branding/footer E2E</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6">
+        <f>COUNTIF('Results (detail)'!$B$2:$B$500,A28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"PASS")</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"OK (recorded)")</f>
+        <v/>
+      </c>
+      <c r="O28" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="P28" s="6">
+        <f>COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"BLOCKED")+COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"NOT RUN")+COUNTIFS('Results (detail)'!$B$2:$B$500,A28,'Results (detail)'!$I$2:$I$500,"ISSUE")</f>
+        <v/>
+      </c>
+      <c r="Q28" s="6" t="inlineStr">
+        <is>
+          <t>PASS with open items</t>
+        </is>
+      </c>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>No real owner upload on production yet (no test data on production) - watch the first one in /admin/document-uploads</t>
+        </is>
+      </c>
+      <c r="S28" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md (15 Oct, production)</t>
         </is>
       </c>
     </row>
@@ -3937,7 +4280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I341"/>
+  <dimension ref="A1:I363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -19137,6 +19480,988 @@
         </is>
       </c>
       <c r="I341" s="6" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="6" t="inlineStr">
+        <is>
+          <t>RES-0341</t>
+        </is>
+      </c>
+      <c r="B342" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C342" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D342" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E342" s="6" t="n"/>
+      <c r="F342" s="6" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="G342" s="6" t="inlineStr">
+        <is>
+          <t>CI 'test' job on PR #169 (full suite + production build)</t>
+        </is>
+      </c>
+      <c r="H342" s="6" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="I342" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="6" t="inlineStr">
+        <is>
+          <t>RES-0342</t>
+        </is>
+      </c>
+      <c r="B343" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C343" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D343" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E343" s="6" t="n"/>
+      <c r="F343" s="6" t="inlineStr">
+        <is>
+          <t>Unit + integration</t>
+        </is>
+      </c>
+      <c r="G343" s="6" t="inlineStr">
+        <is>
+          <t>Full vitest suite, local PostgreSQL 16</t>
+        </is>
+      </c>
+      <c r="H343" s="6" t="inlineStr">
+        <is>
+          <t>1,762 passed in 139 files</t>
+        </is>
+      </c>
+      <c r="I343" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="6" t="inlineStr">
+        <is>
+          <t>RES-0343</t>
+        </is>
+      </c>
+      <c r="B344" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C344" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D344" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E344" s="6" t="n"/>
+      <c r="F344" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G344" s="6" t="inlineStr">
+        <is>
+          <t>Integration document-uploads (incl. 5 new browser-read cases)</t>
+        </is>
+      </c>
+      <c r="H344" s="6" t="inlineStr">
+        <is>
+          <t>21/21</t>
+        </is>
+      </c>
+      <c r="I344" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="6" t="inlineStr">
+        <is>
+          <t>RES-0344</t>
+        </is>
+      </c>
+      <c r="B345" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C345" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D345" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E345" s="6" t="n"/>
+      <c r="F345" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G345" s="6" t="inlineStr">
+        <is>
+          <t>Unit ocr-assets-route: five files served at the installed version; other version / file / path 404</t>
+        </is>
+      </c>
+      <c r="H345" s="6" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="I345" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="6" t="inlineStr">
+        <is>
+          <t>RES-0345</t>
+        </is>
+      </c>
+      <c r="B346" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C346" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D346" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E346" s="6" t="n"/>
+      <c r="F346" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G346" s="6" t="inlineStr">
+        <is>
+          <t>E2E document-browser-read, desktop + Pixel 7: read in the browser (engine browser-tesseract), no CSP violation; fallback to the server with /api/ocr-assets blocked</t>
+        </is>
+      </c>
+      <c r="H346" s="6" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="I346" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="6" t="inlineStr">
+        <is>
+          <t>RES-0346</t>
+        </is>
+      </c>
+      <c r="B347" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C347" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D347" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E347" s="6" t="n"/>
+      <c r="F347" s="6" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G347" s="6" t="inlineStr">
+        <is>
+          <t>E2E branding/footer + smoke, desktop + Pixel 7</t>
+        </is>
+      </c>
+      <c r="H347" s="6" t="inlineStr">
+        <is>
+          <t>30/30</t>
+        </is>
+      </c>
+      <c r="I347" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="6" t="inlineStr">
+        <is>
+          <t>RES-0347</t>
+        </is>
+      </c>
+      <c r="B348" s="6" t="inlineStr">
+        <is>
+          <t>TR-25</t>
+        </is>
+      </c>
+      <c r="C348" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D348" s="6" t="inlineStr">
+        <is>
+          <t>14 Oct, automated</t>
+        </is>
+      </c>
+      <c r="E348" s="6" t="n"/>
+      <c r="F348" s="6" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G348" s="6" t="inlineStr">
+        <is>
+          <t>E2E order lifecycle (regression-items-a-e): order -&gt; accept -&gt; pack -&gt; rider -&gt; delivery code -&gt; delivered, refunds, crons, access control</t>
+        </is>
+      </c>
+      <c r="H348" s="6" t="inlineStr">
+        <is>
+          <t>21/21 (2 stale steps D-20 left out)</t>
+        </is>
+      </c>
+      <c r="I348" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="6" t="inlineStr">
+        <is>
+          <t>RES-0348</t>
+        </is>
+      </c>
+      <c r="B349" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C349" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D349" s="6" t="inlineStr">
+        <is>
+          <t>Staging, before #169 (14 Oct)</t>
+        </is>
+      </c>
+      <c r="E349" s="6" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F349" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G349" s="6" t="inlineStr">
+        <is>
+          <t>FSSAI photo upload on E2E Four Features Bakery (desktop), build before #169</t>
+        </is>
+      </c>
+      <c r="H349" s="6" t="inlineStr">
+        <is>
+          <t>NOT_READ, all fields empty, 31 s - reproduces D-18</t>
+        </is>
+      </c>
+      <c r="I349" s="6" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="6" t="inlineStr">
+        <is>
+          <t>RES-0349</t>
+        </is>
+      </c>
+      <c r="B350" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C350" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D350" s="6" t="inlineStr">
+        <is>
+          <t>Staging, after #169 (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E350" s="6" t="n"/>
+      <c r="F350" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G350" s="6" t="inlineStr">
+        <is>
+          <t>Reader files from /api/ocr-assets and CSP</t>
+        </is>
+      </c>
+      <c r="H350" s="6" t="inlineStr">
+        <is>
+          <t>worker, relaxed-SIMD core and English model all 200; script-src has 'wasm-unsafe-eval'; no CSP violation</t>
+        </is>
+      </c>
+      <c r="I350" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="6" t="inlineStr">
+        <is>
+          <t>RES-0350</t>
+        </is>
+      </c>
+      <c r="B351" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C351" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D351" s="6" t="inlineStr">
+        <is>
+          <t>Staging, after #169 (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E351" s="6" t="n"/>
+      <c r="F351" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G351" s="6" t="inlineStr">
+        <is>
+          <t>FSSAI photo upload, desktop</t>
+        </is>
+      </c>
+      <c r="H351" s="6" t="inlineStr">
+        <is>
+          <t>number 11521998000123, name, expiry 2027-03-31 pre-filled; NAME_MISMATCH warning (expected: the test licence name differs from the owner); 25 s on the first request after deploy, 7.4 s on re-run</t>
+        </is>
+      </c>
+      <c r="I351" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="6" t="inlineStr">
+        <is>
+          <t>RES-0351</t>
+        </is>
+      </c>
+      <c r="B352" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C352" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D352" s="6" t="inlineStr">
+        <is>
+          <t>Staging, after #169 (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E352" s="6" t="n"/>
+      <c r="F352" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G352" s="6" t="inlineStr">
+        <is>
+          <t>FSSAI photo upload, Pixel 7</t>
+        </is>
+      </c>
+      <c r="H352" s="6" t="inlineStr">
+        <is>
+          <t>same fields pre-filled, 8.4 s</t>
+        </is>
+      </c>
+      <c r="I352" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="6" t="inlineStr">
+        <is>
+          <t>RES-0352</t>
+        </is>
+      </c>
+      <c r="B353" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C353" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D353" s="6" t="inlineStr">
+        <is>
+          <t>Staging, after #169 (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E353" s="6" t="n"/>
+      <c r="F353" s="6" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="G353" s="6" t="inlineStr">
+        <is>
+          <t>/admin/document-uploads shows the upload's engine</t>
+        </is>
+      </c>
+      <c r="H353" s="6" t="inlineStr">
+        <is>
+          <t>File · browser-tesseract 92%</t>
+        </is>
+      </c>
+      <c r="I353" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="6" t="inlineStr">
+        <is>
+          <t>RES-0353</t>
+        </is>
+      </c>
+      <c r="B354" s="6" t="inlineStr">
+        <is>
+          <t>TR-26</t>
+        </is>
+      </c>
+      <c r="C354" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D354" s="6" t="inlineStr">
+        <is>
+          <t>Staging, after #169 (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E354" s="6" t="n"/>
+      <c r="F354" s="6" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G354" s="6" t="inlineStr">
+        <is>
+          <t>E2E branding/footer on test.gokesari.com</t>
+        </is>
+      </c>
+      <c r="H354" s="6" t="inlineStr">
+        <is>
+          <t>18/18</t>
+        </is>
+      </c>
+      <c r="I354" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="6" t="inlineStr">
+        <is>
+          <t>RES-0354</t>
+        </is>
+      </c>
+      <c r="B355" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C355" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D355" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E355" s="6" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="F355" s="6" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="G355" s="6" t="inlineStr">
+        <is>
+          <t>Before the release: 8 public pages; /api/ocr-assets; CSP</t>
+        </is>
+      </c>
+      <c r="H355" s="6" t="inlineStr">
+        <is>
+          <t>pages 200; /api/ocr-assets 404; no 'wasm-unsafe-eval' (old build)</t>
+        </is>
+      </c>
+      <c r="I355" s="6" t="inlineStr">
+        <is>
+          <t>OK (recorded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="6" t="inlineStr">
+        <is>
+          <t>RES-0355</t>
+        </is>
+      </c>
+      <c r="B356" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C356" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D356" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E356" s="6" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="F356" s="6" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="G356" s="6" t="inlineStr">
+        <is>
+          <t>New build live on gokesari.com (#175; #177 merged the same commit, no change)</t>
+        </is>
+      </c>
+      <c r="H356" s="6" t="inlineStr">
+        <is>
+          <t>/api/ocr-assets 200</t>
+        </is>
+      </c>
+      <c r="I356" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="6" t="inlineStr">
+        <is>
+          <t>RES-0356</t>
+        </is>
+      </c>
+      <c r="B357" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C357" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D357" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E357" s="6" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F357" s="6" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="G357" s="6" t="inlineStr">
+        <is>
+          <t>/, /shops, /search, /categories, /signin, /sell, /legal/privacy-policy, /api/referral-settings; /shop/documents, /admin/document-uploads signed out</t>
+        </is>
+      </c>
+      <c r="H357" s="6" t="inlineStr">
+        <is>
+          <t>all 200; 307 to sign-in</t>
+        </is>
+      </c>
+      <c r="I357" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="6" t="inlineStr">
+        <is>
+          <t>RES-0357</t>
+        </is>
+      </c>
+      <c r="B358" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C358" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D358" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E358" s="6" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F358" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G358" s="6" t="inlineStr">
+        <is>
+          <t>Five reader files; another version</t>
+        </is>
+      </c>
+      <c r="H358" s="6" t="inlineStr">
+        <is>
+          <t>all 200 (111 KB worker, 3.9 MB cores, 2.9 MB model); other version 404</t>
+        </is>
+      </c>
+      <c r="I358" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="6" t="inlineStr">
+        <is>
+          <t>RES-0358</t>
+        </is>
+      </c>
+      <c r="B359" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C359" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D359" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E359" s="6" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F359" s="6" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="G359" s="6" t="inlineStr">
+        <is>
+          <t>CSP script-src</t>
+        </is>
+      </c>
+      <c r="H359" s="6" t="inlineStr">
+        <is>
+          <t>'wasm-unsafe-eval' present; eval still blocked</t>
+        </is>
+      </c>
+      <c r="I359" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="6" t="inlineStr">
+        <is>
+          <t>RES-0359</t>
+        </is>
+      </c>
+      <c r="B360" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C360" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D360" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E360" s="6" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="F360" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G360" s="6" t="inlineStr">
+        <is>
+          <t>Reader in Chromium on /signin, desktop, from gokesari.com's own files, on an image drawn in the browser (nothing uploaded)</t>
+        </is>
+      </c>
+      <c r="H360" s="6" t="inlineStr">
+        <is>
+          <t>'License Number : 11521998000123 / Valid Upto : 31/03/2027' at 91 %, 3.9 s, no CSP violation</t>
+        </is>
+      </c>
+      <c r="I360" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="6" t="inlineStr">
+        <is>
+          <t>RES-0360</t>
+        </is>
+      </c>
+      <c r="B361" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C361" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D361" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E361" s="6" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="F361" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G361" s="6" t="inlineStr">
+        <is>
+          <t>Same, Pixel 7</t>
+        </is>
+      </c>
+      <c r="H361" s="6" t="inlineStr">
+        <is>
+          <t>same text at 91 %, 2.3 s, no CSP violation</t>
+        </is>
+      </c>
+      <c r="I361" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="6" t="inlineStr">
+        <is>
+          <t>RES-0361</t>
+        </is>
+      </c>
+      <c r="B362" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C362" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D362" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E362" s="6" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F362" s="6" t="inlineStr">
+        <is>
+          <t>Regression</t>
+        </is>
+      </c>
+      <c r="G362" s="6" t="inlineStr">
+        <is>
+          <t>E2E branding/footer on gokesari.com</t>
+        </is>
+      </c>
+      <c r="H362" s="6" t="inlineStr">
+        <is>
+          <t>18/18</t>
+        </is>
+      </c>
+      <c r="I362" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="6" t="inlineStr">
+        <is>
+          <t>RES-0362</t>
+        </is>
+      </c>
+      <c r="B363" s="6" t="inlineStr">
+        <is>
+          <t>TR-27</t>
+        </is>
+      </c>
+      <c r="C363" s="6" t="inlineStr">
+        <is>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md</t>
+        </is>
+      </c>
+      <c r="D363" s="6" t="inlineStr">
+        <is>
+          <t>Production (15 Oct)</t>
+        </is>
+      </c>
+      <c r="E363" s="6" t="n"/>
+      <c r="F363" s="6" t="inlineStr">
+        <is>
+          <t>Document upload</t>
+        </is>
+      </c>
+      <c r="G363" s="6" t="inlineStr">
+        <is>
+          <t>A real shop owner's photo upload on gokesari.com</t>
+        </is>
+      </c>
+      <c r="H363" s="6" t="inlineStr">
+        <is>
+          <t>Not run: no test data on production; watch the first real upload in /admin/document-uploads (engine browser-tesseract)</t>
+        </is>
+      </c>
+      <c r="I363" s="6" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
@@ -19881,17 +21206,17 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>#169 (released via #175 / #177)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Owners type the details; fix tesseract's start or decide on DOCUMENT_OCR_PROVIDER=claude</t>
+          <t>Photos are read in the owner's browser; verified on test (TR-26) and production (TR-27), 15 Oct</t>
         </is>
       </c>
     </row>
@@ -20258,7 +21583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -20594,6 +21919,28 @@
       <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Verified on test</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Real shop-owner photo upload on production with browser reading</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>No test data on production; checked read-only instead (TR-27)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>First real upload, /admin/document-uploads</t>
         </is>
       </c>
     </row>
@@ -21390,6 +22737,7 @@
         <v/>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>

</xml_diff>